<commit_message>
Record the M2 spot check: 16 of 18 points agree (89%)
</commit_message>
<xml_diff>
--- a/docs/m2_spot_check.xlsx
+++ b/docs/m2_spot_check.xlsx
@@ -747,12 +747,20 @@
           <t>Vegetation</t>
         </is>
       </c>
-      <c r="F2" s="8" t="n"/>
+      <c r="F2" s="8" t="inlineStr">
+        <is>
+          <t>Vegetation</t>
+        </is>
+      </c>
       <c r="G2" s="5">
         <f>IF(OR(F2="",F2="Unsure / can't tell"),"",IF(F2=E2,"Yes","No"))</f>
         <v/>
       </c>
-      <c r="H2" s="8" t="n"/>
+      <c r="H2" s="8" t="inlineStr">
+        <is>
+          <t>Grass and trees, International Garden park. [Checked 5 Oct 2026 by Claude (AI assistant) in Google Maps satellite view; Airbus imagery 2026; not blind]</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="n">
@@ -774,12 +782,20 @@
           <t>Bare soil / sand</t>
         </is>
       </c>
-      <c r="F3" s="8" t="n"/>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>Bare soil / sand</t>
+        </is>
+      </c>
       <c r="G3" s="5">
         <f>IF(OR(F3="",F3="Unsure / can't tell"),"",IF(F3=E3,"Yes","No"))</f>
         <v/>
       </c>
-      <c r="H3" s="8" t="n"/>
+      <c r="H3" s="8" t="inlineStr">
+        <is>
+          <t>Open dusty yard beside Seoudi supermarket, cars parked; unpaved-looking (could be dusty paving). [Checked 5 Oct 2026 by Claude (AI assistant) in Google Maps satellite view; Airbus imagery 2026; not blind]</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="n">
@@ -801,12 +817,20 @@
           <t>Bare soil / sand</t>
         </is>
       </c>
-      <c r="F4" s="8" t="n"/>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>Dark surface</t>
+        </is>
+      </c>
       <c r="G4" s="5">
         <f>IF(OR(F4="",F4="Unsure / can't tell"),"",IF(F4=E4,"Yes","No"))</f>
         <v/>
       </c>
-      <c r="H4" s="8" t="n"/>
+      <c r="H4" s="8" t="inlineStr">
+        <is>
+          <t>Carriageway of Ibrahim Shawqi St: dusty grey asphalt next to parked buses. [Checked 5 Oct 2026 by Claude (AI assistant) in Google Maps satellite view; Airbus imagery 2026; not blind]</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="n">
@@ -828,12 +852,20 @@
           <t>Vegetation</t>
         </is>
       </c>
-      <c r="F5" s="8" t="n"/>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>Vegetation</t>
+        </is>
+      </c>
       <c r="G5" s="5">
         <f>IF(OR(F5="",F5="Unsure / can't tell"),"",IF(F5=E5,"Yes","No"))</f>
         <v/>
       </c>
-      <c r="H5" s="8" t="n"/>
+      <c r="H5" s="8" t="inlineStr">
+        <is>
+          <t>Tree canopy in a walled garden plot. [Checked 5 Oct 2026 by Claude (AI assistant) in Google Maps satellite view; Airbus imagery 2026; not blind]</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="n">
@@ -855,12 +887,20 @@
           <t>Dark surface</t>
         </is>
       </c>
-      <c r="F6" s="8" t="n"/>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>Dark surface</t>
+        </is>
+      </c>
       <c r="G6" s="5">
         <f>IF(OR(F6="",F6="Unsure / can't tell"),"",IF(F6=E6,"Yes","No"))</f>
         <v/>
       </c>
-      <c r="H6" s="8" t="n"/>
+      <c r="H6" s="8" t="inlineStr">
+        <is>
+          <t>Asphalt carriageway, Mostafa El-Nahaas St. [Checked 5 Oct 2026 by Claude (AI assistant) in Google Maps satellite view; Airbus imagery 2026; not blind]</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="n">
@@ -882,12 +922,20 @@
           <t>Dark surface</t>
         </is>
       </c>
-      <c r="F7" s="8" t="n"/>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>Dark surface</t>
+        </is>
+      </c>
       <c r="G7" s="5">
         <f>IF(OR(F7="",F7="Unsure / can't tell"),"",IF(F7=E7,"Yes","No"))</f>
         <v/>
       </c>
-      <c r="H7" s="8" t="n"/>
+      <c r="H7" s="8" t="inlineStr">
+        <is>
+          <t>Asphalt carriageway, Abd Allah El-Araby St. [Checked 5 Oct 2026 by Claude (AI assistant) in Google Maps satellite view; Airbus imagery 2026; not blind]</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="n">
@@ -909,12 +957,20 @@
           <t>Bright surface</t>
         </is>
       </c>
-      <c r="F8" s="8" t="n"/>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>Unsure / can't tell</t>
+        </is>
+      </c>
       <c r="G8" s="5">
         <f>IF(OR(F8="",F8="Unsure / can't tell"),"",IF(F8=E8,"Yes","No"))</f>
         <v/>
       </c>
-      <c r="H8" s="8" t="n"/>
+      <c r="H8" s="8" t="inlineStr">
+        <is>
+          <t>Narrow dusty strip between a tree hedge and a small building; mixed within 10 m. [Checked 5 Oct 2026 by Claude (AI assistant) in Google Maps satellite view; Airbus imagery 2026; not blind]</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="n">
@@ -936,12 +992,20 @@
           <t>Vegetation</t>
         </is>
       </c>
-      <c r="F9" s="8" t="n"/>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>Vegetation</t>
+        </is>
+      </c>
       <c r="G9" s="5">
         <f>IF(OR(F9="",F9="Unsure / can't tell"),"",IF(F9=E9,"Yes","No"))</f>
         <v/>
       </c>
-      <c r="H9" s="8" t="n"/>
+      <c r="H9" s="8" t="inlineStr">
+        <is>
+          <t>Edge of tree canopy and a sandy path in a small tree park (mostly trees). [Checked 5 Oct 2026 by Claude (AI assistant) in Google Maps satellite view; Airbus imagery 2026; not blind]</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="n">
@@ -963,12 +1027,20 @@
           <t>Bare soil / sand</t>
         </is>
       </c>
-      <c r="F10" s="8" t="n"/>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>Bright surface</t>
+        </is>
+      </c>
       <c r="G10" s="5">
         <f>IF(OR(F10="",F10="Unsure / can't tell"),"",IF(F10=E10,"Yes","No"))</f>
         <v/>
       </c>
-      <c r="H10" s="8" t="n"/>
+      <c r="H10" s="8" t="inlineStr">
+        <is>
+          <t>Dusty beige concrete rooftop (inside a building footprint). [Checked 5 Oct 2026 by Claude (AI assistant) in Google Maps satellite view; Airbus imagery 2026; not blind]</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="n">
@@ -990,12 +1062,20 @@
           <t>Bare soil / sand</t>
         </is>
       </c>
-      <c r="F11" s="8" t="n"/>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>Bare soil / sand</t>
+        </is>
+      </c>
       <c r="G11" s="5">
         <f>IF(OR(F11="",F11="Unsure / can't tell"),"",IF(F11=E11,"Yes","No"))</f>
         <v/>
       </c>
-      <c r="H11" s="8" t="n"/>
+      <c r="H11" s="8" t="inlineStr">
+        <is>
+          <t>Large vacant sandy lot, just inside its southern wall. [Checked 5 Oct 2026 by Claude (AI assistant) in Google Maps satellite view; Airbus imagery 2026; not blind]</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="n">
@@ -1017,12 +1097,20 @@
           <t>Bright surface</t>
         </is>
       </c>
-      <c r="F12" s="8" t="n"/>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>Bright surface</t>
+        </is>
+      </c>
       <c r="G12" s="5">
         <f>IF(OR(F12="",F12="Unsure / can't tell"),"",IF(F12=E12,"Yes","No"))</f>
         <v/>
       </c>
-      <c r="H12" s="8" t="n"/>
+      <c r="H12" s="8" t="inlineStr">
+        <is>
+          <t>Pale concrete rooftops, on the edge between two roofs. [Checked 5 Oct 2026 by Claude (AI assistant) in Google Maps satellite view; Airbus imagery 2026; not blind]</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="n">
@@ -1044,12 +1132,20 @@
           <t>Vegetation</t>
         </is>
       </c>
-      <c r="F13" s="8" t="n"/>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>Vegetation</t>
+        </is>
+      </c>
       <c r="G13" s="5">
         <f>IF(OR(F13="",F13="Unsure / can't tell"),"",IF(F13=E13,"Yes","No"))</f>
         <v/>
       </c>
-      <c r="H13" s="8" t="n"/>
+      <c r="H13" s="8" t="inlineStr">
+        <is>
+          <t>Grass and trees in a park. [Checked 5 Oct 2026 by Claude (AI assistant) in Google Maps satellite view; Airbus imagery 2026; not blind]</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="n">
@@ -1071,12 +1167,20 @@
           <t>Dark surface</t>
         </is>
       </c>
-      <c r="F14" s="8" t="n"/>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>Dark surface</t>
+        </is>
+      </c>
       <c r="G14" s="5">
         <f>IF(OR(F14="",F14="Unsure / can't tell"),"",IF(F14=E14,"Yes","No"))</f>
         <v/>
       </c>
-      <c r="H14" s="8" t="n"/>
+      <c r="H14" s="8" t="inlineStr">
+        <is>
+          <t>Asphalt carriageway, Mostafa El-Nahaas St. [Checked 5 Oct 2026 by Claude (AI assistant) in Google Maps satellite view; Airbus imagery 2026; not blind]</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="n">
@@ -1098,12 +1202,20 @@
           <t>Bare soil / sand</t>
         </is>
       </c>
-      <c r="F15" s="8" t="n"/>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>Bare soil / sand</t>
+        </is>
+      </c>
       <c r="G15" s="5">
         <f>IF(OR(F15="",F15="Unsure / can't tell"),"",IF(F15=E15,"Yes","No"))</f>
         <v/>
       </c>
-      <c r="H15" s="8" t="n"/>
+      <c r="H15" s="8" t="inlineStr">
+        <is>
+          <t>Unpaved dirt ground beside a road ramp, vehicles parked on it. [Checked 5 Oct 2026 by Claude (AI assistant) in Google Maps satellite view; Airbus imagery 2026; not blind]</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="n">
@@ -1125,12 +1237,20 @@
           <t>Vegetation</t>
         </is>
       </c>
-      <c r="F16" s="8" t="n"/>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>Vegetation</t>
+        </is>
+      </c>
       <c r="G16" s="5">
         <f>IF(OR(F16="",F16="Unsure / can't tell"),"",IF(F16=E16,"Yes","No"))</f>
         <v/>
       </c>
-      <c r="H16" s="8" t="n"/>
+      <c r="H16" s="8" t="inlineStr">
+        <is>
+          <t>Dense tree canopy in a park. [Checked 5 Oct 2026 by Claude (AI assistant) in Google Maps satellite view; Airbus imagery 2026; not blind]</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="n">
@@ -1152,12 +1272,20 @@
           <t>Bright surface</t>
         </is>
       </c>
-      <c r="F17" s="8" t="n"/>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>Bright surface</t>
+        </is>
+      </c>
       <c r="G17" s="5">
         <f>IF(OR(F17="",F17="Unsure / can't tell"),"",IF(F17=E17,"Yes","No"))</f>
         <v/>
       </c>
-      <c r="H17" s="8" t="n"/>
+      <c r="H17" s="8" t="inlineStr">
+        <is>
+          <t>Pale concrete rooftop. [Checked 5 Oct 2026 by Claude (AI assistant) in Google Maps satellite view; Airbus imagery 2026; not blind]</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="n">
@@ -1179,12 +1307,20 @@
           <t>Dark surface</t>
         </is>
       </c>
-      <c r="F18" s="8" t="n"/>
+      <c r="F18" s="8" t="inlineStr">
+        <is>
+          <t>Dark surface</t>
+        </is>
+      </c>
       <c r="G18" s="5">
         <f>IF(OR(F18="",F18="Unsure / can't tell"),"",IF(F18=E18,"Yes","No"))</f>
         <v/>
       </c>
-      <c r="H18" s="8" t="n"/>
+      <c r="H18" s="8" t="inlineStr">
+        <is>
+          <t>Asphalt carriageway, El Tayaran St. [Checked 5 Oct 2026 by Claude (AI assistant) in Google Maps satellite view; Airbus imagery 2026; not blind]</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="n">
@@ -1206,12 +1342,20 @@
           <t>Bright surface</t>
         </is>
       </c>
-      <c r="F19" s="8" t="n"/>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>Bright surface</t>
+        </is>
+      </c>
       <c r="G19" s="5">
         <f>IF(OR(F19="",F19="Unsure / can't tell"),"",IF(F19=E19,"Yes","No"))</f>
         <v/>
       </c>
-      <c r="H19" s="8" t="n"/>
+      <c r="H19" s="8" t="inlineStr">
+        <is>
+          <t>Pale paved sidewalk between a building and Mohammed Hussein Haykal St (edge). [Checked 5 Oct 2026 by Claude (AI assistant) in Google Maps satellite view; Airbus imagery 2026; not blind]</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="n">
@@ -1233,12 +1377,20 @@
           <t>Bright surface</t>
         </is>
       </c>
-      <c r="F20" s="8" t="n"/>
+      <c r="F20" s="8" t="inlineStr">
+        <is>
+          <t>Unsure / can't tell</t>
+        </is>
+      </c>
       <c r="G20" s="5">
         <f>IF(OR(F20="",F20="Unsure / can't tell"),"",IF(F20=E20,"Yes","No"))</f>
         <v/>
       </c>
-      <c r="H20" s="8" t="n"/>
+      <c r="H20" s="8" t="inlineStr">
+        <is>
+          <t>Deep shadow in a narrow gap between two buildings; material not visible. [Checked 5 Oct 2026 by Claude (AI assistant) in Google Maps satellite view; Airbus imagery 2026; not blind]</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="n">
@@ -1260,12 +1412,20 @@
           <t>Dark surface</t>
         </is>
       </c>
-      <c r="F21" s="8" t="n"/>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>Dark surface</t>
+        </is>
+      </c>
       <c r="G21" s="5">
         <f>IF(OR(F21="",F21="Unsure / can't tell"),"",IF(F21=E21,"Yes","No"))</f>
         <v/>
       </c>
-      <c r="H21" s="8" t="n"/>
+      <c r="H21" s="8" t="inlineStr">
+        <is>
+          <t>Asphalt carriageway, El Tayaran St. [Checked 5 Oct 2026 by Claude (AI assistant) in Google Maps satellite view; Airbus imagery 2026; not blind]</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="9" t="inlineStr">

</xml_diff>